<commit_message>
Update annotations, YouTube fetcher, and frame annotation scripts
</commit_message>
<xml_diff>
--- a/annotations/Final/preprocessed_dataset_1_FULL_STATS.xlsx
+++ b/annotations/Final/preprocessed_dataset_1_FULL_STATS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\a9188\Documents\00. 2024 QMUL\00. Course\Project\00. ViolenceDetectionProject\annotations\Final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6067E870-A10F-4F1E-AF77-98D2E4B73E2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D17F9F4-E544-4FE7-9608-DB9C19405278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -167,9 +167,6 @@
     </r>
   </si>
   <si>
-    <t>Final violence detection dataset – v1 statistics</t>
-  </si>
-  <si>
     <t>Modality</t>
   </si>
   <si>
@@ -186,6 +183,9 @@
   </si>
   <si>
     <t>⊙ Modality</t>
+  </si>
+  <si>
+    <t>Final violence detection dataset statistics</t>
   </si>
 </sst>
 </file>
@@ -356,6 +356,72 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>110434</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>248478</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>533952</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>100219</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="그림 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AF920F0D-44DF-78F6-A700-35F6B904DC00}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="10861260" y="408608"/>
+          <a:ext cx="8926996" cy="3816350"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -665,7 +731,7 @@
   <sheetData>
     <row r="2" spans="2:14" ht="30" customHeight="1">
       <c r="B2" s="13" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C2" s="13"/>
       <c r="D2" s="13"/>
@@ -688,7 +754,7 @@
         <v>34</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="2:14" ht="13">
@@ -708,7 +774,7 @@
         <v>18</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="M6" s="3" t="s">
         <v>6</v>
@@ -765,7 +831,7 @@
         <v>0.61273666092943202</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="M8" s="10">
         <v>1523</v>
@@ -787,7 +853,7 @@
         <v>0.25430292598967297</v>
       </c>
       <c r="L9" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="M9" s="10">
         <v>555</v>
@@ -809,7 +875,7 @@
         <v>0.13296041308089501</v>
       </c>
       <c r="L10" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="M10" s="10">
         <v>223</v>
@@ -821,7 +887,7 @@
     </row>
     <row r="11" spans="2:14">
       <c r="L11" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M11" s="10">
         <v>23</v>
@@ -1000,6 +1066,7 @@
     <mergeCell ref="B2:N2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>